<commit_message>
Automate monthly evidence updates
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_final_combined.xlsx
+++ b/Plot/exposures_meta_analysis_final_combined.xlsx
@@ -2828,34 +2828,34 @@
         </is>
       </c>
       <c r="B68" s="4" t="n">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>1.41</v>
+        <v>1.38</v>
       </c>
       <c r="D68" s="5" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>1.46</v>
+        <v>1.44</v>
       </c>
       <c r="F68" s="5" t="n">
         <v>0.87</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>2.26</v>
+        <v>2.2</v>
       </c>
       <c r="H68" s="6" t="n">
         <v>98.2</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>8.121947612144099e-07</v>
+        <v>5.91216845462099e-07</v>
       </c>
       <c r="J68" s="8" t="n">
-        <v>15616182</v>
+        <v>17027950</v>
       </c>
       <c r="K68" s="8" t="n">
-        <v>1431464</v>
+        <v>1688752</v>
       </c>
     </row>
     <row r="69">

</xml_diff>